<commit_message>
Update Master BOM details: updated 51 front wiring part numbers across 391 vehicle codes
</commit_message>
<xml_diff>
--- a/Bom details.xlsx
+++ b/Bom details.xlsx
@@ -4912,7 +4912,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>547854600152</t>
+          <t>547854600226</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -4956,7 +4956,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>547854600152</t>
+          <t>547854600226</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -5000,7 +5000,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>547854600178</t>
+          <t>547854600267</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -5022,7 +5022,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>547854600122</t>
+          <t>547854600269</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -5044,7 +5044,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>547854600268</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -5066,7 +5066,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>547854600210</t>
+          <t>547854600270</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -5110,7 +5110,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>547854600120</t>
+          <t>547854600223</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -5154,7 +5154,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>547854600121</t>
+          <t>547854600224</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -5198,7 +5198,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>547854600121</t>
+          <t>547854600224</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -5242,7 +5242,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>547854600118</t>
+          <t>547854600222</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -5286,7 +5286,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>547854600118</t>
+          <t>547854600222</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -5308,7 +5308,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>547854600209</t>
+          <t>547854600268</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -5330,7 +5330,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>547854600210</t>
+          <t>547854600270</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -5352,7 +5352,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>547854600209</t>
+          <t>547854600268</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -5374,7 +5374,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>547854600210</t>
+          <t>547854600270</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -5462,7 +5462,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>547854600268</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -5506,7 +5506,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>547854600178</t>
+          <t>547854600267</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -5528,7 +5528,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>547854600122</t>
+          <t>547854600269</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -5572,7 +5572,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>547854600120</t>
+          <t>547854600223</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>547854600152</t>
+          <t>547854600226</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -5682,7 +5682,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>547854600152</t>
+          <t>547854600226</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -5704,7 +5704,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>547854600178</t>
+          <t>547854600267</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -5726,7 +5726,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>547854600122</t>
+          <t>547854600269</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -5748,7 +5748,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>547854600178</t>
+          <t>547854600267</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -5770,7 +5770,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>547854600122</t>
+          <t>547854600269</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -5792,7 +5792,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>547854600178</t>
+          <t>547854600267</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>547854600122</t>
+          <t>547854600269</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -5836,7 +5836,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>547854600178</t>
+          <t>547854600267</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -5858,7 +5858,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>547854600122</t>
+          <t>547854600269</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -5880,7 +5880,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>547854600209</t>
+          <t>547854600268</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -5902,7 +5902,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>547854600210</t>
+          <t>547854600270</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -5924,7 +5924,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>547854600268</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -5968,7 +5968,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>547854600209</t>
+          <t>547854600268</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -5990,7 +5990,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>547854600210</t>
+          <t>547854600270</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -6034,7 +6034,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>547854600121</t>
+          <t>547854600224</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -6078,7 +6078,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>547854600121</t>
+          <t>547854600224</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -6122,7 +6122,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>547854600172</t>
+          <t>547854600227</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -6166,7 +6166,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>547854600172</t>
+          <t>547854600227</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -6188,7 +6188,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>DATA Not found</t>
+          <t>547854600267</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -6210,7 +6210,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>DATA Not found</t>
+          <t>547854600269</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -6232,7 +6232,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>DATA Not found</t>
+          <t>547854600267</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
@@ -6254,7 +6254,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>547854600269</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -6276,7 +6276,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>547854600209</t>
+          <t>547854600268</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -6298,7 +6298,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>547854600210</t>
+          <t>547854600270</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -6320,7 +6320,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>547854600268</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>547854600268</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -6474,7 +6474,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>DATA Not found</t>
+          <t>547854600270</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -6496,7 +6496,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>547854600268</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -6518,7 +6518,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>547854600210</t>
+          <t>547854600270</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -6540,7 +6540,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>547854600268</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -6606,7 +6606,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>DATA Not found</t>
+          <t>547854600270</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">

</xml_diff>